<commit_message>
Migrate Performance & Portfolio chapter (code + charts)
- import-performance.js reuses the chapter-page template with autoAccordion
  (sections transformer now derives accordion sub-chapters from the DOM
  instead of hardcoded ids), plus chapter-nav / callout-case-study / logo-grid
- Rasterized 11 oversized (>20KB) infographic charts to PNG under assets/charts
  and extended the cleanup transformer's SVG->PNG remap
- chapter-cleanup collapses DataTables scroll-widget duplicates to the single
  real table

Note: the interactive DataTables (esp. 30-row Major Investments) are accepted
as-is for now per scope; 2 div-tables still mis-parse but are non-fatal.
Content is authored to DA separately.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-chapter-page.report.xlsx
+++ b/tools/importer/reports/import-chapter-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,6 +37,30 @@
     <t>url</t>
   </si>
   <si>
+    <t>from-our-chairman.report.json</t>
+  </si>
+  <si>
+    <t>["columns-feature"]</t>
+  </si>
+  <si>
+    <t>from-our-chairman</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>letter-page</t>
+  </si>
+  <si>
+    <t>2026-07-08T17:59:27.046Z</t>
+  </si>
+  <si>
+    <t>From Our Chairman | Temasek Review 2026</t>
+  </si>
+  <si>
+    <t>https://www.temasekreview.com.sg/from-our-chairman.html</t>
+  </si>
+  <si>
     <t>index.report.json</t>
   </si>
   <si>
@@ -46,9 +70,6 @@
     <t>index</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>homepage</t>
   </si>
   <si>
@@ -64,7 +85,7 @@
     <t>strategy.report.json</t>
   </si>
   <si>
-    <t>["callout-case-study","callout-case-study","callout-case-study","callout-case-study","logo-grid","logo-grid","logo-grid"]</t>
+    <t>["chapter-nav","callout-case-study","callout-case-study","callout-case-study","callout-case-study","logo-grid","logo-grid","logo-grid"]</t>
   </si>
   <si>
     <t>strategy</t>
@@ -73,7 +94,7 @@
     <t>chapter-page</t>
   </si>
   <si>
-    <t>2026-07-08T17:18:27.256Z</t>
+    <t>2026-07-09T05:11:06.201Z</t>
   </si>
   <si>
     <t>Strategy | Temasek Review 2026</t>
@@ -468,16 +489,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="1" max="1" width="31" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="3" max="3" width="19" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="49" customWidth="1"/>
-    <col min="8" max="8" width="48" customWidth="1"/>
+    <col min="8" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -556,6 +577,32 @@
       </c>
       <c r="H3" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>